<commit_message>
Track 1 methods form: record the three additions with their measurements
Rows 9, 14, 16, 18 and 19 updated. The compound-heterozygote question (row 16)
now describes phase elimination as a filter with its numbers, the public-data
row names the alignment reference and the gnomAD API queries, run time includes
the 4h35 read-level analysis, and the abstract states the background count, the
lowered mosaicism floor, and the limitation that bulk coverage is structurally
blind to variegated aneuploidy.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VeqGJD7TYQeozqCSqdL4WX
</commit_message>
<xml_diff>
--- a/submissions/henkvaness_track1_methods_model1.xlsx
+++ b/submissions/henkvaness_track1_methods_model1.xlsx
@@ -527,7 +527,6 @@
     </row>
     <row r="3"/>
     <row r="4"/>
-    <row r="5"/>
     <row r="6" ht="16" customHeight="1" s="7">
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -567,7 +566,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Scripted pipeline (pipeline/run.sh, 61 s): PASS variants in BUB1B/CEP57/TRIP13 annotated offline with bcftools csq (Ensembl 116) and ClinVar; gnomAD v4.1 counts by HTTP range read; genome-wide recessive-compatible scan without gene list; mosaic aneuploidy profile from allele depths; ACMG SF v3.2 screen; CSV built by a written scoring rule (make_csv.py) and checked against the Space's scorer. Full report: REPORT_track1.md.</t>
+          <t>Scripted pipeline (pipeline/run.sh, 61 s): PASS variants in BUB1B/CEP57/TRIP13 annotated offline with bcftools csq (Ensembl 116) and ClinVar; gnomAD v4.1 counts by HTTP range read; genome-wide recessive-compatible scan without gene list; mosaic aneuploidy profile from allele depths; ACMG SF v3.2 screen; CSV built by a written scoring rule (make_csv.py) and checked against the Space's scorer. Three later additions, each recorded with its measurement: (a) the candidate's own rarity threshold applied to the whole genome, so the background is measured on the same criterion rather than a proxy (8 genes reach AF &lt; 1e-4 on both variants, 2 reach AF &lt; 1e-5); (b) read-backed phase (PGT/PID) used as an eliminator across all candidate genes rather than as a check on one, removing 79 of 151 genes in the wide grouping and 3 of the 8 above; (c) the supplied raw reads aligned and coverage measured in 100 kb windows with GC-bin normalisation, which lowers the mosaic-aneuploidy detection floor from about 10% to about 4% of cells. Full report: REPORT_track1.md; the three additions are R15, R16 and R17 in track2/reanalysis/.</t>
         </is>
       </c>
     </row>
@@ -627,7 +626,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Ensembl release 116 GFF3 and GRCh38 FASTA; ClinVar GRCh38 VCF (5 Sep 2026); gnomAD v4.1 exome and genome sites (chr15); ACMG SF v3.2 gene list; OMIM 257300 and published BUB1B literature for interpretation.</t>
+          <t>Ensembl release 116 GFF3 and GRCh38 FASTA; GRCh38 no-alt analysis set (the reference the supplied VCF was called against), used for read alignment; ClinVar GRCh38 VCF (5 Sep 2026); gnomAD v4.1 exome and genome sites, read by HTTP range for chr15 and by the public gnomAD API for the genome-wide background (876 variants queried, 850 returned); ACMG SF v3.2 gene list; OMIM 257300 and published BUB1B literature for interpretation.</t>
         </is>
       </c>
     </row>
@@ -651,7 +650,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Yes: the top two heterozygous candidates in one gene are submitted as a pair (row 1), each alone (rows 2-3), then alternative pairings.</t>
+          <t>Yes: the top two heterozygous candidates in one gene are submitted as a pair (row 1), each alone (rows 2-3), then alternative pairings. Candidate pairs are additionally filtered on read-backed phase: where both variants of a gene sit in the same GATK phase set (PID) with the same orientation (PGT) they are on one haplotype, the other allele is intact, and the gene is eliminated by evidence rather than by argument. This removes 79 of the 151 genes carrying two rare heterozygous coding variants, and 3 of the 8 that meet the candidate's own frequency threshold, including KIR3DL3, the only other gene at AF &lt; 1e-5. It cannot resolve BUB1B itself: its two variants are 10,911 bp apart, far beyond fragment length, so phase there remains unproven and requires parental genotyping or long reads.</t>
         </is>
       </c>
     </row>
@@ -675,7 +674,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>61 seconds on a laptop (single process), about 1 GB of public reference downloads, no cloud compute, no paid API.</t>
+          <t>Core pipeline: 61 seconds on a laptop (single process), about 1 GB of public reference downloads, no cloud compute, no paid API. The optional read-level analysis is the expensive part: 78.85 GB of supplied FASTQ downloaded, aligned with minimap2 on a 20-core server in 4 h 35 min wall clock, 137 GB peak disk, median coverage 51x. Raw reads and alignments are deleted after the hackathon under the data use terms.</t>
         </is>
       </c>
     </row>
@@ -687,7 +686,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>A one-minute, fully scripted pipeline recovers a compound-heterozygous BUB1B genotype (p.Leu737Ter, ClinVar pathogenic; p.Asn1002Lys, gnomAD singleton) from a standard germline VCF, confirms rarity from gnomAD without exporting any query, screens ACMG secondary findings, and quantifies mosaic aneuploidy from the same file with a stated detection floor. Limitations: the known-gene pass is disease-specific; the genome-wide check lacks population frequencies and phenotype scoring (Exomiser planned); phase cannot be established without parents or long reads; structural variants and deep intronic variants are not evaluated; the mosaicism method is blind to balanced rearrangements and to mosaicism below about 10%.</t>
+          <t>A one-minute, fully scripted pipeline recovers a compound-heterozygous BUB1B genotype (p.Leu737Ter, ClinVar pathogenic; p.Asn1002Lys, gnomAD singleton) from a standard germline VCF, confirms rarity from gnomAD, screens ACMG secondary findings, and quantifies mosaic aneuploidy from the same file. Three additions strengthen the evidence rather than the answer. First, the background is measured on the candidate's own criterion: 8 genes in this genome carry two variants at AF &lt; 1e-4, and 2 at AF &lt; 1e-5, so the compound-heterozygous pattern is specific but not unique, and the case rests on frequency plus consequence plus phenotype rather than on the pattern alone. Second, read-backed phase is used as an eliminator across all candidates, not as a check on one, removing 79 of 151 genes with proof, including the candidate's nearest competitor. Third, the supplied raw reads were aligned and coverage measured in 100 kb windows with GC-bin normalisation, lowering the mosaic-aneuploidy floor from about 10% to about 4% of cells; nothing is present above it, and chrX at 0.498 and chrY at 0.512 confirm the sex configuration independently of genotypes. Limitations, stated rather than discovered: phase for BUB1B cannot be established without parents or long reads, and no amount of re-processing changes that; structural and deep intronic variants are not evaluated; the known-gene pass is disease-specific and the panel was implied by the supplied phenotype document, which names chromosomal instability disorders; and the coverage method is structurally blind to this phenotype, because variegated aneuploidy places different chromosomes in different cells, so the per-chromosome affected fraction falls far below any bulk floor. That last point is why karyotyping remains the diagnostic standard here and why sequencing cannot replace it.</t>
         </is>
       </c>
     </row>

</xml_diff>